<commit_message>
refactor: Renomei uma coluna na base de perícias
</commit_message>
<xml_diff>
--- a/app/data/db_character_skills.xlsx
+++ b/app/data/db_character_skills.xlsx
@@ -34,7 +34,7 @@
     <t>skill_difficulty</t>
   </si>
   <si>
-    <t>skill_base_status</t>
+    <t>skill_base_attribute</t>
   </si>
   <si>
     <t>skill_pre_defined_level</t>
@@ -3003,7 +3003,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">

</xml_diff>